<commit_message>
Reconcile Table 3 and Supplementary Table S4 with identical inclusion criteria and cancer-type stratified Cox
</commit_message>
<xml_diff>
--- a/results/Table 3.xlsx
+++ b/results/Table 3.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total (N)</t>
+          <t>Total Analyzed (N)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -478,246 +478,246 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCEC</t>
+          <t>BLCA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Uterine Corpus Endometrial Carcinoma</t>
+          <t>Bladder Urothelial Carcinoma</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>475</v>
+        <v>433</v>
       </c>
       <c r="D2" t="n">
-        <v>142</v>
+        <v>107</v>
       </c>
       <c r="E2" t="n">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.43 (0.24 - 0.77)</t>
+          <t>0.67 (0.47 - 0.94)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.0045</t>
+          <t>0.0224</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.64 (0.29 - 1.42)</t>
+          <t>0.89 (0.60 - 1.30)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.2741</t>
+          <t>0.5359</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BLCA</t>
+          <t>BRCA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bladder Urothelial Carcinoma</t>
+          <t>Breast Invasive Carcinoma</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>433</v>
+        <v>913</v>
       </c>
       <c r="D3" t="n">
-        <v>107</v>
+        <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>326</v>
+        <v>863</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.67 (0.47 - 0.94)</t>
+          <t>0.79 (0.35 - 1.80)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.0224</t>
+          <t>0.5731</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.89 (0.60 - 1.30)</t>
+          <t>0.66 (0.28 - 1.53)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.5359</t>
+          <t>0.3318</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>STAD</t>
+          <t>COAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Stomach Adenocarcinoma</t>
+          <t>Colon Adenocarcinoma</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>468</v>
+        <v>331</v>
       </c>
       <c r="D4" t="n">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="E4" t="n">
-        <v>361</v>
+        <v>250</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.69 (0.48 - 0.99)</t>
+          <t>1.11 (0.70 - 1.77)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.0421</t>
+          <t>0.6534</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.82 (0.53 - 1.27)</t>
+          <t>0.95 (0.53 - 1.71)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.3798</t>
+          <t>0.8611</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LUAD</t>
+          <t>HNSC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lung Adenocarcinoma</t>
+          <t>Head and Neck Squamous Cell Carcinoma</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>622</v>
+        <v>582</v>
       </c>
       <c r="D5" t="n">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>528</v>
+        <v>510</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.71 (0.48 - 1.05)</t>
+          <t>0.74 (0.49 - 1.10)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.0864</t>
+          <t>0.1308</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.68 (0.45 - 1.04)</t>
+          <t>0.66 (0.44 - 0.99)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.0729</t>
+          <t>0.0447</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HNSC</t>
+          <t>KIRC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Head and Neck Squamous Cell Carcinoma</t>
+          <t>Kidney Renal Clear Cell Carcinoma</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>582</v>
+        <v>626</v>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="E6" t="n">
-        <v>510</v>
+        <v>595</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.74 (0.49 - 1.10)</t>
+          <t>1.98 (1.15 - 3.42)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.1308</t>
+          <t>0.0138</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.66 (0.44 - 0.99)</t>
+          <t>1.13 (0.60 - 2.13)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.0447</t>
+          <t>0.7000</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>LUAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Breast Invasive Carcinoma</t>
+          <t>Lung Adenocarcinoma</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>913</v>
+        <v>622</v>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="E7" t="n">
-        <v>863</v>
+        <v>528</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.79 (0.35 - 1.80)</t>
+          <t>0.71 (0.48 - 1.05)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.5731</t>
+          <t>0.0864</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.66 (0.28 - 1.53)</t>
+          <t>0.68 (0.45 - 1.04)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.3318</t>
+          <t>0.0729</t>
         </is>
       </c>
     </row>
@@ -765,123 +765,123 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COAD</t>
+          <t>SKCM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Colon Adenocarcinoma</t>
+          <t>Skin Cutaneous Melanoma</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>331</v>
+        <v>458</v>
       </c>
       <c r="D9" t="n">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="E9" t="n">
-        <v>250</v>
+        <v>305</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1.11 (0.70 - 1.77)</t>
+          <t>1.16 (0.88 - 1.54)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.6534</t>
+          <t>0.2860</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.95 (0.53 - 1.71)</t>
+          <t>1.55 (1.14 - 2.11)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.8611</t>
+          <t>0.0055</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SKCM</t>
+          <t>STAD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Skin Cutaneous Melanoma</t>
+          <t>Stomach Adenocarcinoma</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="D10" t="n">
-        <v>153</v>
+        <v>107</v>
       </c>
       <c r="E10" t="n">
-        <v>305</v>
+        <v>361</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1.16 (0.88 - 1.54)</t>
+          <t>0.69 (0.48 - 0.99)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.2860</t>
+          <t>0.0421</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1.55 (1.14 - 2.11)</t>
+          <t>0.82 (0.53 - 1.27)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0.0055</t>
+          <t>0.3798</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KIRC</t>
+          <t>UCEC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kidney Renal Clear Cell Carcinoma</t>
+          <t>Uterine Corpus Endometrial Carcinoma</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>626</v>
+        <v>475</v>
       </c>
       <c r="D11" t="n">
-        <v>31</v>
+        <v>142</v>
       </c>
       <c r="E11" t="n">
-        <v>595</v>
+        <v>333</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.98 (1.15 - 3.42)</t>
+          <t>0.43 (0.24 - 0.77)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.0138</t>
+          <t>0.0045</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.13 (0.60 - 2.13)</t>
+          <t>0.64 (0.29 - 1.42)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.7000</t>
+          <t>0.2741</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Combined TCGA Pan-Cancer Cohort</t>
+          <t>Combined TCGA Pan-Cancer Cohort (Cancer-Type Stratified)</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -907,22 +907,22 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.08 (0.97 - 1.20)</t>
+          <t>0.87 (0.78 - 0.98)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.1514</t>
+          <t>0.0167</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.67 (0.59 - 0.76)</t>
+          <t>0.87 (0.77 - 0.98)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>&lt; 0.0001</t>
+          <t>0.0188</t>
         </is>
       </c>
     </row>

</xml_diff>